<commit_message>
updating functions / cleanup code
</commit_message>
<xml_diff>
--- a/test/export/Fathom_Deployment_Data_Sheet_GMY_2025.xlsx
+++ b/test/export/Fathom_Deployment_Data_Sheet_GMY_2025.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -402,26 +402,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Frankland_reef</t>
+          <t>Scotts Reef</t>
         </is>
       </c>
       <c r="B2" s="2">
-        <v>45627.03125</v>
+        <v>45605.17361111111</v>
       </c>
       <c r="C2" s="2">
-        <v>45940.06944444445</v>
+        <v>45959.10069444445</v>
       </c>
       <c r="D2">
-        <v>-17.2105</v>
+        <v>-17.058195</v>
       </c>
       <c r="E2">
-        <v>146.07424</v>
+        <v>146.178219</v>
       </c>
       <c r="F2">
-        <v>127282</v>
+        <v>491823</v>
       </c>
       <c r="G2">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -456,7 +456,10 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <v>45940.02777777778</v>
+        <v>45627.03125</v>
+      </c>
+      <c r="C4" s="2">
+        <v>45940.06944444445</v>
       </c>
       <c r="D4">
         <v>-17.2105</v>
@@ -465,7 +468,7 @@
         <v>146.07424</v>
       </c>
       <c r="F4">
-        <v>137057</v>
+        <v>127282</v>
       </c>
       <c r="G4">
         <v>14</v>
@@ -491,6 +494,50 @@
       </c>
       <c r="G5">
         <v>12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Frankland_reef</t>
+        </is>
+      </c>
+      <c r="B6" s="2">
+        <v>45940.02777777778</v>
+      </c>
+      <c r="D6">
+        <v>-17.2105</v>
+      </c>
+      <c r="E6">
+        <v>146.07424</v>
+      </c>
+      <c r="F6">
+        <v>137057</v>
+      </c>
+      <c r="G6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Scotts Reef</t>
+        </is>
+      </c>
+      <c r="B7" s="2">
+        <v>45959.10069444445</v>
+      </c>
+      <c r="D7">
+        <v>-17.058195</v>
+      </c>
+      <c r="E7">
+        <v>146.178219</v>
+      </c>
+      <c r="F7">
+        <v>136066</v>
+      </c>
+      <c r="G7">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>